<commit_message>
Updates to periods as per the claude identified conflcits
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanwin/Documents/NallamSchools/NRHS/Time Table/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanwin/Documents/GitHub/School_TimeTable/NRHS/Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFCA118F-ABE6-B343-A89A-2C4BABAD8DE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2B41FC-AE59-0D4B-8B02-E10C1B631A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{09F5BE17-A93C-C440-BF2B-7788082B8849}"/>
+    <workbookView xWindow="-28800" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="1" xr2:uid="{09F5BE17-A93C-C440-BF2B-7788082B8849}"/>
   </bookViews>
   <sheets>
     <sheet name="Teacher Allotment" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="84">
   <si>
     <t>TELUGU</t>
   </si>
@@ -290,13 +290,16 @@
   </si>
   <si>
     <t>1(A)</t>
+  </si>
+  <si>
+    <t>Total Periods</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -376,6 +379,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -401,7 +411,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -433,53 +443,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -517,23 +487,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1139,7 +1100,7 @@
         <v>13</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G10" s="11"/>
       <c r="H10" s="11"/>
@@ -1516,13 +1477,13 @@
         <v>7</v>
       </c>
       <c r="H5" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I5" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J5" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K5" s="3">
         <v>6</v>
@@ -1870,196 +1831,257 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="3">
         <v>3</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="3">
         <v>3</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="3">
         <v>3</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="3">
         <v>3</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="3">
         <v>3</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="3">
         <v>4</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="3">
+        <v>2</v>
+      </c>
+      <c r="I13" s="3">
+        <v>2</v>
+      </c>
+      <c r="J13" s="3">
+        <v>2</v>
+      </c>
+      <c r="K13" s="3">
         <v>1</v>
       </c>
-      <c r="I13" s="5">
+      <c r="L13" s="3">
         <v>1</v>
       </c>
-      <c r="J13" s="5">
+      <c r="M13" s="3">
         <v>1</v>
       </c>
-      <c r="K13" s="5">
+      <c r="N13" s="3">
         <v>1</v>
       </c>
-      <c r="L13" s="5">
+      <c r="O13" s="3">
         <v>1</v>
       </c>
-      <c r="M13" s="5">
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="3">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>2</v>
+      </c>
+      <c r="F14" s="3">
+        <v>2</v>
+      </c>
+      <c r="G14" s="3">
+        <v>2</v>
+      </c>
+      <c r="H14" s="3">
         <v>1</v>
       </c>
-      <c r="N13" s="5">
+      <c r="I14" s="3">
         <v>1</v>
       </c>
-      <c r="O13" s="19">
+      <c r="J14" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A14" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" s="5">
-        <v>0</v>
-      </c>
-      <c r="C14" s="5">
-        <v>0</v>
-      </c>
-      <c r="D14" s="5">
-        <v>0</v>
-      </c>
-      <c r="E14" s="5">
-        <v>2</v>
-      </c>
-      <c r="F14" s="5">
-        <v>2</v>
-      </c>
-      <c r="G14" s="5">
-        <v>2</v>
-      </c>
-      <c r="H14" s="5">
+      <c r="K14" s="3">
         <v>1</v>
       </c>
-      <c r="I14" s="5">
+      <c r="L14" s="3">
         <v>1</v>
       </c>
-      <c r="J14" s="5">
+      <c r="M14" s="3">
         <v>1</v>
       </c>
-      <c r="K14" s="5">
+      <c r="N14" s="3">
+        <v>0</v>
+      </c>
+      <c r="O14" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="16">
+        <v>6</v>
+      </c>
+      <c r="C15" s="16">
+        <v>6</v>
+      </c>
+      <c r="D15" s="16">
+        <v>6</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3">
+        <v>0</v>
+      </c>
+      <c r="J15" s="3">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3">
+        <v>0</v>
+      </c>
+      <c r="L15" s="3">
+        <v>0</v>
+      </c>
+      <c r="M15" s="3">
+        <v>0</v>
+      </c>
+      <c r="N15" s="3">
+        <v>0</v>
+      </c>
+      <c r="O15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3">
         <v>1</v>
       </c>
-      <c r="L14" s="5">
+      <c r="F16" s="3">
         <v>1</v>
       </c>
-      <c r="M14" s="5">
+      <c r="G16" s="3">
         <v>1</v>
       </c>
-      <c r="N14" s="5">
-        <v>0</v>
-      </c>
-      <c r="O14" s="19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A15" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B15" s="15">
-        <v>6</v>
-      </c>
-      <c r="C15" s="15">
-        <v>6</v>
-      </c>
-      <c r="D15" s="15">
-        <v>6</v>
-      </c>
-      <c r="E15" s="5">
-        <v>0</v>
-      </c>
-      <c r="F15" s="5">
-        <v>0</v>
-      </c>
-      <c r="G15" s="5">
-        <v>0</v>
-      </c>
-      <c r="H15" s="5">
-        <v>0</v>
-      </c>
-      <c r="I15" s="5">
-        <v>0</v>
-      </c>
-      <c r="J15" s="5">
-        <v>0</v>
-      </c>
-      <c r="K15" s="5">
-        <v>0</v>
-      </c>
-      <c r="L15" s="5">
-        <v>0</v>
-      </c>
-      <c r="M15" s="5">
-        <v>0</v>
-      </c>
-      <c r="N15" s="5">
-        <v>0</v>
-      </c>
-      <c r="O15" s="19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A16" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="B16" s="16">
-        <v>0</v>
-      </c>
-      <c r="C16" s="16">
-        <v>0</v>
-      </c>
-      <c r="D16" s="16">
-        <v>0</v>
-      </c>
-      <c r="E16" s="16">
+      <c r="H16" s="3">
         <v>1</v>
       </c>
-      <c r="F16" s="16">
+      <c r="I16" s="3">
         <v>1</v>
       </c>
-      <c r="G16" s="16">
+      <c r="J16" s="3">
         <v>1</v>
       </c>
-      <c r="H16" s="16">
+      <c r="K16" s="3">
         <v>1</v>
       </c>
-      <c r="I16" s="16">
+      <c r="L16" s="3">
         <v>1</v>
       </c>
-      <c r="J16" s="16">
+      <c r="M16" s="3">
         <v>1</v>
       </c>
-      <c r="K16" s="16">
-        <v>1</v>
-      </c>
-      <c r="L16" s="16">
-        <v>1</v>
-      </c>
-      <c r="M16" s="16">
-        <v>1</v>
-      </c>
-      <c r="N16" s="16">
-        <v>0</v>
-      </c>
-      <c r="O16" s="21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="N16" s="3">
+        <v>0</v>
+      </c>
+      <c r="O16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="18">
+        <f>SUM(B3:B16)</f>
+        <v>42</v>
+      </c>
+      <c r="C17" s="18">
+        <f t="shared" ref="C17:O17" si="0">SUM(C3:C16)</f>
+        <v>42</v>
+      </c>
+      <c r="D17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="E17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="F17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="G17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="H17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="I17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="J17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="K17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="L17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="M17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="N17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="O17" s="18">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="C21" s="14"/>
-      <c r="D21" s="17"/>
+      <c r="D21" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Changes to time table
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanwin/Documents/GitHub/School_TimeTable/NRHS/Requirements/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanwin/Documents/NallamSchools/NRHS/Time Table/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2B41FC-AE59-0D4B-8B02-E10C1B631A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{923FD2E2-BE51-0648-9214-BEDB6AE16CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28800" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="1" xr2:uid="{09F5BE17-A93C-C440-BF2B-7788082B8849}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="86">
   <si>
     <t>TELUGU</t>
   </si>
@@ -292,14 +292,20 @@
     <t>1(A)</t>
   </si>
   <si>
-    <t>Total Periods</t>
+    <t>S.GAYATRI</t>
+  </si>
+  <si>
+    <t>SUMANI</t>
+  </si>
+  <si>
+    <t>Study Hour</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -379,13 +385,6 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFC00000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -411,7 +410,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -443,13 +442,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -487,14 +526,29 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -833,10 +887,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11520368-A10D-A341-8FD4-4B05F59ACE8F}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -870,8 +924,11 @@
       <c r="K1" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L1" s="22" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>21</v>
       </c>
@@ -893,8 +950,9 @@
       <c r="I2" s="11"/>
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" s="23"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>64</v>
       </c>
@@ -918,8 +976,9 @@
       <c r="I3" s="11"/>
       <c r="J3" s="11"/>
       <c r="K3" s="11"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L3" s="23"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>74</v>
       </c>
@@ -943,8 +1002,9 @@
       <c r="I4" s="11"/>
       <c r="J4" s="11"/>
       <c r="K4" s="11"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" s="23"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>65</v>
       </c>
@@ -970,8 +1030,11 @@
       <c r="K5" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L5" s="23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>66</v>
       </c>
@@ -997,8 +1060,11 @@
       <c r="K6" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L6" s="23" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>33</v>
       </c>
@@ -1024,8 +1090,11 @@
       <c r="K7" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L7" s="23" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -1053,8 +1122,11 @@
       <c r="K8" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L8" s="23" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>35</v>
       </c>
@@ -1082,8 +1154,11 @@
       <c r="K9" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>36</v>
       </c>
@@ -1100,7 +1175,7 @@
         <v>13</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G10" s="11"/>
       <c r="H10" s="11"/>
@@ -1111,8 +1186,11 @@
       <c r="K10" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>37</v>
       </c>
@@ -1144,8 +1222,11 @@
       <c r="K11" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>38</v>
       </c>
@@ -1177,8 +1258,11 @@
       <c r="K12" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>39</v>
       </c>
@@ -1210,8 +1294,11 @@
       <c r="K13" s="11" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>40</v>
       </c>
@@ -1241,8 +1328,9 @@
         <v>16</v>
       </c>
       <c r="K14" s="11"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" s="23"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>41</v>
       </c>
@@ -1272,8 +1360,9 @@
         <v>16</v>
       </c>
       <c r="K15" s="11"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L15" s="23"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="12"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
@@ -1285,8 +1374,9 @@
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" s="12"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1298,6 +1388,7 @@
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1477,13 +1568,13 @@
         <v>7</v>
       </c>
       <c r="H5" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I5" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J5" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K5" s="3">
         <v>6</v>
@@ -1527,10 +1618,10 @@
         <v>7</v>
       </c>
       <c r="I6" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J6" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K6" s="3">
         <v>6</v>
@@ -1831,257 +1922,196 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="5">
         <v>3</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="5">
         <v>3</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="5">
         <v>3</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="5">
         <v>3</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="5">
         <v>3</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="5">
         <v>4</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="5">
+        <v>1</v>
+      </c>
+      <c r="I13" s="5">
         <v>2</v>
       </c>
-      <c r="I13" s="3">
+      <c r="J13" s="5">
         <v>2</v>
       </c>
-      <c r="J13" s="3">
+      <c r="K13" s="5">
+        <v>1</v>
+      </c>
+      <c r="L13" s="5">
+        <v>1</v>
+      </c>
+      <c r="M13" s="5">
+        <v>1</v>
+      </c>
+      <c r="N13" s="5">
+        <v>1</v>
+      </c>
+      <c r="O13" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A14" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="5">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5">
         <v>2</v>
       </c>
-      <c r="K13" s="3">
+      <c r="F14" s="5">
+        <v>2</v>
+      </c>
+      <c r="G14" s="5">
+        <v>2</v>
+      </c>
+      <c r="H14" s="5">
         <v>1</v>
       </c>
-      <c r="L13" s="3">
+      <c r="I14" s="5">
         <v>1</v>
       </c>
-      <c r="M13" s="3">
+      <c r="J14" s="5">
         <v>1</v>
       </c>
-      <c r="N13" s="3">
+      <c r="K14" s="5">
         <v>1</v>
       </c>
-      <c r="O13" s="3">
+      <c r="L14" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" s="3">
-        <v>0</v>
-      </c>
-      <c r="C14" s="3">
-        <v>0</v>
-      </c>
-      <c r="D14" s="3">
-        <v>0</v>
-      </c>
-      <c r="E14" s="3">
-        <v>2</v>
-      </c>
-      <c r="F14" s="3">
-        <v>2</v>
-      </c>
-      <c r="G14" s="3">
-        <v>2</v>
-      </c>
-      <c r="H14" s="3">
+      <c r="M14" s="5">
         <v>1</v>
       </c>
-      <c r="I14" s="3">
+      <c r="N14" s="5">
+        <v>0</v>
+      </c>
+      <c r="O14" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A15" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="15">
+        <v>6</v>
+      </c>
+      <c r="C15" s="15">
+        <v>6</v>
+      </c>
+      <c r="D15" s="15">
+        <v>6</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5">
+        <v>0</v>
+      </c>
+      <c r="K15" s="5">
+        <v>0</v>
+      </c>
+      <c r="L15" s="5">
+        <v>0</v>
+      </c>
+      <c r="M15" s="5">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5">
+        <v>0</v>
+      </c>
+      <c r="O15" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A16" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="16">
+        <v>0</v>
+      </c>
+      <c r="C16" s="16">
+        <v>0</v>
+      </c>
+      <c r="D16" s="16">
+        <v>0</v>
+      </c>
+      <c r="E16" s="16">
         <v>1</v>
       </c>
-      <c r="J14" s="3">
+      <c r="F16" s="16">
         <v>1</v>
       </c>
-      <c r="K14" s="3">
+      <c r="G16" s="16">
         <v>1</v>
       </c>
-      <c r="L14" s="3">
+      <c r="H16" s="16">
         <v>1</v>
       </c>
-      <c r="M14" s="3">
+      <c r="I16" s="16">
         <v>1</v>
       </c>
-      <c r="N14" s="3">
-        <v>0</v>
-      </c>
-      <c r="O14" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B15" s="16">
-        <v>6</v>
-      </c>
-      <c r="C15" s="16">
-        <v>6</v>
-      </c>
-      <c r="D15" s="16">
-        <v>6</v>
-      </c>
-      <c r="E15" s="3">
-        <v>0</v>
-      </c>
-      <c r="F15" s="3">
-        <v>0</v>
-      </c>
-      <c r="G15" s="3">
-        <v>0</v>
-      </c>
-      <c r="H15" s="3">
-        <v>0</v>
-      </c>
-      <c r="I15" s="3">
-        <v>0</v>
-      </c>
-      <c r="J15" s="3">
-        <v>0</v>
-      </c>
-      <c r="K15" s="3">
-        <v>0</v>
-      </c>
-      <c r="L15" s="3">
-        <v>0</v>
-      </c>
-      <c r="M15" s="3">
-        <v>0</v>
-      </c>
-      <c r="N15" s="3">
-        <v>0</v>
-      </c>
-      <c r="O15" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B16" s="3">
-        <v>0</v>
-      </c>
-      <c r="C16" s="3">
-        <v>0</v>
-      </c>
-      <c r="D16" s="3">
-        <v>0</v>
-      </c>
-      <c r="E16" s="3">
+      <c r="J16" s="16">
         <v>1</v>
       </c>
-      <c r="F16" s="3">
+      <c r="K16" s="16">
         <v>1</v>
       </c>
-      <c r="G16" s="3">
+      <c r="L16" s="16">
         <v>1</v>
       </c>
-      <c r="H16" s="3">
+      <c r="M16" s="16">
         <v>1</v>
       </c>
-      <c r="I16" s="3">
-        <v>1</v>
-      </c>
-      <c r="J16" s="3">
-        <v>1</v>
-      </c>
-      <c r="K16" s="3">
-        <v>1</v>
-      </c>
-      <c r="L16" s="3">
-        <v>1</v>
-      </c>
-      <c r="M16" s="3">
-        <v>1</v>
-      </c>
-      <c r="N16" s="3">
-        <v>0</v>
-      </c>
-      <c r="O16" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="B17" s="18">
-        <f>SUM(B3:B16)</f>
-        <v>42</v>
-      </c>
-      <c r="C17" s="18">
-        <f t="shared" ref="C17:O17" si="0">SUM(C3:C16)</f>
-        <v>42</v>
-      </c>
-      <c r="D17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="E17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="F17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="G17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="H17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="I17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="J17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="K17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="L17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="M17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="N17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="O17" s="18">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N16" s="16">
+        <v>0</v>
+      </c>
+      <c r="O16" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C21" s="14"/>
-      <c r="D21" s="15"/>
+      <c r="D21" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2090,7 +2120,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC79E649-3C05-194C-B9BA-F0ABC9C3A63B}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -2190,6 +2220,44 @@
         <v>79</v>
       </c>
     </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (19 Jul 2026 22:22)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-60" yWindow="-60" windowWidth="21720" windowHeight="12900" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Weekly Period Plan" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,14 +14,14 @@
     <sheet name="Activity Plan" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,81 +29,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Aptos"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF7030A0"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.5999938962981048"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002A4D69"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="7">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -110,130 +46,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -597,921 +418,878 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O18"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.796875" defaultRowHeight="14.25"/>
-  <cols>
-    <col width="12.86328125" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
-    <col width="6" customWidth="1" style="1" min="2" max="2"/>
-    <col width="8.33203125" customWidth="1" style="1" min="3" max="3"/>
-    <col width="9" customWidth="1" style="1" min="4" max="4"/>
-    <col width="10.06640625" customWidth="1" style="1" min="5" max="5"/>
-    <col width="11.265625" customWidth="1" style="1" min="6" max="6"/>
-    <col width="7.1328125" bestFit="1" customWidth="1" style="1" min="7" max="14"/>
-    <col width="7.86328125" bestFit="1" customWidth="1" style="1" min="15" max="15"/>
-    <col width="8.796875" customWidth="1" style="1" min="16" max="16384"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Weekly Period Plan</t>
         </is>
       </c>
-      <c r="B1" s="19" t="n"/>
-      <c r="C1" s="19" t="n"/>
-      <c r="D1" s="19" t="n"/>
-      <c r="E1" s="19" t="n"/>
-      <c r="F1" s="19" t="n"/>
-      <c r="G1" s="19" t="n"/>
-      <c r="H1" s="19" t="n"/>
-      <c r="I1" s="19" t="n"/>
-      <c r="J1" s="19" t="n"/>
-      <c r="K1" s="19" t="n"/>
-      <c r="L1" s="19" t="n"/>
-      <c r="M1" s="19" t="n"/>
-      <c r="N1" s="19" t="n"/>
-      <c r="O1" s="20" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>LKG</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>UKG(A)</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>UKG(B)</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Class 1(A)</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Class 1(B)</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Class 2</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Class 3</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Class 4</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Class 5</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Class 6</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Class 7</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Class 8</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Class 9</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Class 10</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Telugu</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" t="n">
         <v>5</v>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N3" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O3" s="4" t="n">
+      <c r="C3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>6</v>
+      </c>
+      <c r="K3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L3" t="n">
+        <v>6</v>
+      </c>
+      <c r="M3" t="n">
+        <v>6</v>
+      </c>
+      <c r="N3" t="n">
+        <v>6</v>
+      </c>
+      <c r="O3" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Hindi</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="4" t="n">
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" t="n">
         <v>5</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" t="n">
         <v>5</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" t="n">
         <v>5</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" t="n">
         <v>5</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" t="n">
         <v>5</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" t="n">
         <v>5</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M4" t="n">
         <v>5</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" t="n">
         <v>8</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" t="n">
         <v>8</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K5" s="4" t="n">
+      <c r="E5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" t="n">
         <v>5</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="L5" t="n">
         <v>5</v>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="M5" t="n">
         <v>5</v>
       </c>
-      <c r="N5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O5" s="4" t="n">
+      <c r="N5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O5" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Eng Grammar</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4" t="n">
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="K6" t="n">
         <v>1</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="L6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="M6" t="n">
         <v>1</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="O6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Maths</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" t="n">
         <v>10</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" t="n">
         <v>7</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" t="n">
         <v>7</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" t="n">
         <v>7</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" t="n">
         <v>7</v>
       </c>
-      <c r="I7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M7" s="4" t="n">
+      <c r="I7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" t="n">
+        <v>6</v>
+      </c>
+      <c r="K7" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" t="n">
         <v>7</v>
       </c>
-      <c r="N7" s="4" t="n">
+      <c r="N7" t="n">
         <v>8</v>
       </c>
-      <c r="O7" s="4" t="n">
+      <c r="O7" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>EVS</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" t="n">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" t="n">
         <v>7</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" t="n">
         <v>7</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" t="n">
         <v>7</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" t="n">
         <v>7</v>
       </c>
-      <c r="H8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="4" t="n">
+      <c r="H8" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="4" t="n">
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
         <v>2</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="L9" t="n">
         <v>2</v>
       </c>
-      <c r="M9" s="4" t="n">
+      <c r="M9" t="n">
         <v>4</v>
       </c>
-      <c r="N9" s="4" t="n">
+      <c r="N9" t="n">
         <v>5</v>
       </c>
-      <c r="O9" s="4" t="n">
+      <c r="O9" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="4" t="n">
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
         <v>3</v>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="L10" t="n">
         <v>3</v>
       </c>
-      <c r="M10" s="4" t="n">
+      <c r="M10" t="n">
         <v>4</v>
       </c>
-      <c r="N10" s="4" t="n">
+      <c r="N10" t="n">
         <v>4</v>
       </c>
-      <c r="O10" s="4" t="n">
+      <c r="O10" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="4" t="n">
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
         <v>3</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="L11" t="n">
         <v>3</v>
       </c>
-      <c r="M11" s="4" t="n">
+      <c r="M11" t="n">
         <v>4</v>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="N11" t="n">
         <v>4</v>
       </c>
-      <c r="O11" s="4" t="n">
+      <c r="O11" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Social</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O12" s="4" t="n">
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" t="n">
+        <v>6</v>
+      </c>
+      <c r="K12" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" t="n">
+        <v>6</v>
+      </c>
+      <c r="M12" t="n">
+        <v>6</v>
+      </c>
+      <c r="N12" t="n">
+        <v>6</v>
+      </c>
+      <c r="O12" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Computer</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="4" t="n">
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="H13" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="I13" t="n">
         <v>2</v>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="J13" t="n">
         <v>2</v>
       </c>
-      <c r="K13" s="4" t="n">
+      <c r="K13" t="n">
         <v>2</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="L13" t="n">
         <v>2</v>
       </c>
-      <c r="M13" s="4" t="n">
+      <c r="M13" t="n">
         <v>2</v>
       </c>
-      <c r="N13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="4" t="n">
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>P.E.T</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="F14" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="H14" t="n">
         <v>2</v>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="I14" t="n">
         <v>2</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="J14" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="4" t="n">
+      <c r="K14" t="n">
         <v>2</v>
       </c>
-      <c r="L14" s="4" t="n">
+      <c r="L14" t="n">
         <v>2</v>
       </c>
-      <c r="M14" s="4" t="n">
+      <c r="M14" t="n">
         <v>2</v>
       </c>
-      <c r="N14" s="4" t="n">
+      <c r="N14" t="n">
         <v>2</v>
       </c>
-      <c r="O14" s="4" t="n">
+      <c r="O14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>G.K</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="4" t="n">
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" t="n">
         <v>2</v>
       </c>
-      <c r="H15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="4" t="n">
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
         <v>1</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="J15" t="n">
         <v>1</v>
       </c>
-      <c r="K15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="4" t="n">
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Oral</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="4" t="n">
+      <c r="B16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Karate</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="4" t="n">
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="G17" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="H17" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="I17" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="J17" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="4" t="n">
+      <c r="K17" t="n">
         <v>1</v>
       </c>
-      <c r="L17" s="4" t="n">
+      <c r="L17" t="n">
         <v>1</v>
       </c>
-      <c r="M17" s="4" t="n">
+      <c r="M17" t="n">
         <v>1</v>
       </c>
-      <c r="N17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="4" t="n">
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B18" s="8">
-        <f>SUM(B3:B17)</f>
-        <v/>
-      </c>
-      <c r="C18" s="8">
-        <f>SUM(C3:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="8">
-        <f>SUM(D3:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="8">
-        <f>SUM(E3:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="8">
-        <f>SUM(F3:F17)</f>
-        <v/>
-      </c>
-      <c r="G18" s="8">
-        <f>SUM(G3:G17)</f>
-        <v/>
-      </c>
-      <c r="H18" s="8">
-        <f>SUM(H3:H17)</f>
-        <v/>
-      </c>
-      <c r="I18" s="8">
-        <f>SUM(I3:I17)</f>
-        <v/>
-      </c>
-      <c r="J18" s="8">
-        <f>SUM(J3:J17)</f>
-        <v/>
-      </c>
-      <c r="K18" s="8">
-        <f>SUM(K3:K17)</f>
-        <v/>
-      </c>
-      <c r="L18" s="8">
-        <f>SUM(L3:L17)</f>
-        <v/>
-      </c>
-      <c r="M18" s="8">
-        <f>SUM(M3:M17)</f>
-        <v/>
-      </c>
-      <c r="N18" s="8">
-        <f>SUM(N3:N17)</f>
-        <v/>
-      </c>
-      <c r="O18" s="8">
-        <f>SUM(O3:O17)</f>
-        <v/>
+      <c r="B18" t="n">
+        <v>42</v>
+      </c>
+      <c r="C18" t="n">
+        <v>42</v>
+      </c>
+      <c r="D18" t="n">
+        <v>42</v>
+      </c>
+      <c r="E18" t="n">
+        <v>42</v>
+      </c>
+      <c r="F18" t="n">
+        <v>42</v>
+      </c>
+      <c r="G18" t="n">
+        <v>42</v>
+      </c>
+      <c r="H18" t="n">
+        <v>42</v>
+      </c>
+      <c r="I18" t="n">
+        <v>42</v>
+      </c>
+      <c r="J18" t="n">
+        <v>42</v>
+      </c>
+      <c r="K18" t="n">
+        <v>42</v>
+      </c>
+      <c r="L18" t="n">
+        <v>42</v>
+      </c>
+      <c r="M18" t="n">
+        <v>47</v>
+      </c>
+      <c r="N18" t="n">
+        <v>47</v>
+      </c>
+      <c r="O18" t="n">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -1522,769 +1300,744 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.796875" defaultRowHeight="14.25"/>
-  <cols>
-    <col width="11.265625" bestFit="1" customWidth="1" style="9" min="1" max="1"/>
-    <col width="14.19921875" bestFit="1" customWidth="1" style="1" min="2" max="5"/>
-    <col width="11.06640625" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
-    <col width="14.1328125" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
-    <col width="11.86328125" bestFit="1" customWidth="1" style="1" min="8" max="10"/>
-    <col width="11.1328125" bestFit="1" customWidth="1" style="1" min="11" max="12"/>
-    <col width="11.796875" bestFit="1" customWidth="1" style="1" min="13" max="13"/>
-    <col width="12.19921875" bestFit="1" customWidth="1" style="1" min="14" max="15"/>
-    <col width="8.796875" customWidth="1" style="1" min="16" max="16384"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Teacher Allotment</t>
         </is>
       </c>
-      <c r="B1" s="19" t="n"/>
-      <c r="C1" s="19" t="n"/>
-      <c r="D1" s="19" t="n"/>
-      <c r="E1" s="19" t="n"/>
-      <c r="F1" s="19" t="n"/>
-      <c r="G1" s="19" t="n"/>
-      <c r="H1" s="19" t="n"/>
-      <c r="I1" s="19" t="n"/>
-      <c r="J1" s="19" t="n"/>
-      <c r="K1" s="19" t="n"/>
-      <c r="L1" s="20" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>CLASS</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>L.K.G</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>U.K.G(A)</t>
         </is>
       </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>U.K.G(B)</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Class 1(A)</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Class 1(B)</t>
         </is>
       </c>
-      <c r="G2" s="18" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Class 2</t>
         </is>
       </c>
-      <c r="H2" s="18" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Class 3</t>
         </is>
       </c>
-      <c r="I2" s="18" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Class 4</t>
         </is>
       </c>
-      <c r="J2" s="18" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Class 5</t>
         </is>
       </c>
-      <c r="K2" s="18" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Class 6</t>
         </is>
       </c>
-      <c r="L2" s="18" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Class 7</t>
         </is>
       </c>
-      <c r="M2" s="18" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Class 8</t>
         </is>
       </c>
-      <c r="N2" s="18" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Class 9</t>
         </is>
       </c>
-      <c r="O2" s="18" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Class 10</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>TELUGU</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>MAHA LAKSHMI</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>MAHA LAKSHMI</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>MAHA LAKSHMI</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>MAHA LAKSHMI</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>SURYA DEVI</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>P.SATYAVENI</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>P.SATYAVENI</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>P.SATYAVENI</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>P.SATYAVENI</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>M.LALITHA</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>M.LALITHA</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>M.LALITHA</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>M.LALITHA</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>M.LALITHA</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>HINDI</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
         <is>
           <t>BIJILI</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>JAYA LAKSHMI</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>SURYA DEVI</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>SHEKINA</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>SAI KEERTHI</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>SAI KEERTHI</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>SAI KEERTHI</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>SAI KEERTHI</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>SAI KEERTHI</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>RIYA</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>RIYA</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>RIYA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>ENGLISH</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>SHEKINA</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>BIJILI</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>JAYA LAKSHMI</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>SURYA DEVI</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>N.NAVYA</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>N.NAVYA</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>N.NAVYA</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>N.NAVYA</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>N.NAVYA</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>D.SUMANI</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>D.SUMANI</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>D.SUMANI</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>D.SUMANI</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>MATHS</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>SHEKINA</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>BIJILI</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>JAYA LAKSHMI</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>SURYA DEVI</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>S.GAYATHRI</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>CHANDINI</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>CHANDINI</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>CHANDINI</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>CHANDINI</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>CHANDINI</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>D.GOWTHAM</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>D.GOWTHAM</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>EVS</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>SHEKINA</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>BIJILI</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>JAYA LAKSHMI</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>SURYA DEVI</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>JAYA LAKSHMI</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>S.GAYATHRI</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>S.GAYATHRI</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="n"/>
-      <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4" t="n"/>
-      <c r="O7" s="4" t="n"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>PHYSICS</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
-      <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>SAIRAM</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>SAIRAM</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>CHEMISTRY</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
-      <c r="H9" s="4" t="n"/>
-      <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="n"/>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>BIOLOGY</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
-      <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="n"/>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
         <is>
           <t>S.GAYATHRI</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>S.GAYATHRI</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>CHALAPATHI</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>CHALAPATHI</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>CHALAPATHI</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>SOCIAL</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
         <is>
           <t>R.KAMALA</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>R.KAMALA</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>R.KAMALA</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>R.KAMALA</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>R.KAMALA</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>SUNITHA</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>SUNITHA</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>SUNITHA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>COMPUTER</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="N12" s="4" t="n"/>
-      <c r="O12" s="4" t="n"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>G.K</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>SURYA DEVI</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>SATYAVENI</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>NAVYA</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>SAI KEERTHI</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>ESWAR</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>ESWAR</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>CHANDINI</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>ESWAR</t>
         </is>
       </c>
-      <c r="N13" s="4" t="n"/>
-      <c r="O13" s="4" t="n"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2296,266 +2049,235 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.796875" defaultRowHeight="14.25"/>
-  <cols>
-    <col width="15.53125" bestFit="1" customWidth="1" style="9" min="1" max="1"/>
-    <col width="8.796875" customWidth="1" style="1" min="2" max="3"/>
-    <col width="12.33203125" bestFit="1" customWidth="1" style="1" min="4" max="4"/>
-    <col width="10.46484375" customWidth="1" style="1" min="5" max="5"/>
-    <col width="10.33203125" customWidth="1" style="1" min="6" max="6"/>
-    <col width="9" customWidth="1" style="1" min="7" max="7"/>
-    <col width="8.796875" customWidth="1" style="1" min="8" max="8"/>
-    <col width="9.33203125" customWidth="1" style="1" min="9" max="9"/>
-    <col width="9.1328125" customWidth="1" style="1" min="10" max="10"/>
-    <col width="12.33203125" customWidth="1" style="1" min="11" max="11"/>
-    <col width="9.33203125" customWidth="1" style="1" min="12" max="12"/>
-    <col width="8.796875" customWidth="1" style="1" min="13" max="16384"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Period 1 Teacher Allotment</t>
         </is>
       </c>
-      <c r="B1" s="21" t="n"/>
-      <c r="C1" s="21" t="n"/>
-      <c r="D1" s="21" t="n"/>
-      <c r="E1" s="21" t="n"/>
-      <c r="F1" s="21" t="n"/>
-      <c r="G1" s="21" t="n"/>
-      <c r="H1" s="21" t="n"/>
-      <c r="I1" s="21" t="n"/>
-      <c r="J1" s="21" t="n"/>
-      <c r="K1" s="21" t="n"/>
-      <c r="L1" s="21" t="n"/>
-      <c r="M1" s="21" t="n"/>
-      <c r="N1" s="21" t="n"/>
-      <c r="O1" s="21" t="n"/>
-    </row>
-    <row r="2" customFormat="1" s="10">
-      <c r="A2" s="3" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>L.K.G</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>U.K.G 1</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>U.K.G 2</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Class 1(A)</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Class 1(B)</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Class 2</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Class 3</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Class 4</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Class 5</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Class 6</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Class 7</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Class 8</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Class 9</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Class 10</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Period 1 Teacher</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Shekina</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Bijili</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Maha Lakshmi</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Chandrakala</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Surya Devi</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Satyaveni</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Navya</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Sai Keerthi</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Gayatri</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kamala Devi     </t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Kamala Devi</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>Chandini</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Eswari</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lalitha </t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Lalitha</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>Sumani</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Study Hour</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Shekina</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Bijili</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Maha Lakshmi</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Chandrakala</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Surya Devi</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Satyaveni</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Navya</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Sai Keerthi</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Eswari</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kamala Devi     </t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Kamala Devi</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>Chandini</t>
         </is>
       </c>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="4" t="n"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2567,675 +2289,654 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K22"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="10.6640625" defaultRowHeight="14.25"/>
-  <cols>
-    <col width="14.19921875" customWidth="1" style="1" min="1" max="1"/>
-    <col width="15.796875" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
-    <col width="8" bestFit="1" customWidth="1" style="1" min="3" max="6"/>
-    <col width="11.86328125" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
-    <col width="8" bestFit="1" customWidth="1" style="1" min="8" max="10"/>
-    <col width="10.6640625" customWidth="1" style="1" min="11" max="16384"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Teacher Leisure Plan</t>
         </is>
       </c>
-      <c r="B1" s="21" t="n"/>
-      <c r="C1" s="21" t="n"/>
-      <c r="D1" s="21" t="n"/>
-      <c r="E1" s="21" t="n"/>
-      <c r="F1" s="21" t="n"/>
-      <c r="G1" s="21" t="n"/>
-      <c r="H1" s="21" t="n"/>
-      <c r="I1" s="21" t="n"/>
-      <c r="J1" s="21" t="n"/>
-      <c r="K1" s="21" t="n"/>
-    </row>
-    <row r="2" customFormat="1" s="11">
-      <c r="A2" s="12" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Teacher Name</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Leisure Fitmenet</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Leisure Fitment</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Period 1</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Period 2</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Period 3</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Period 4</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Period 5</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Period 6</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Period 7</t>
         </is>
       </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Study Hour</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>RIYA</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>SUNITHA</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>CHALAPATHI</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>D.GOWTHAM</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Leisure</t>
         </is>
       </c>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="n"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>SHEKINA</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H7" s="4" t="n"/>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="n"/>
-      <c r="K7" s="4" t="n"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>BIJILI</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H8" s="4" t="n"/>
-      <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>MAHA LAKSHMI</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H9" s="4" t="n"/>
-      <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="n"/>
-      <c r="K9" s="4" t="n"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H10" s="4" t="n"/>
-      <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="n"/>
-      <c r="K10" s="4" t="n"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>SURYA DEVI</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H11" s="4" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
-      <c r="K11" s="4" t="n"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>M.LALITHA</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="n"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>P.SATYAVENI</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="4" t="n"/>
-      <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>N.NAVYA</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>S.GAYATHRI</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H15" s="4" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
-      <c r="K15" s="4" t="n"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>SAI KEERTHI</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="4" t="n"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>R.KAMALA</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H17" s="4" t="n"/>
-      <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="n"/>
-      <c r="K17" s="4" t="n"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>D.SUMANI</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="n"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>SAIRAM</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>CHANDINI</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="n"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>K,ESWAR</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>K.ESWAR</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H21" s="4" t="n"/>
-      <c r="I21" s="4" t="n"/>
-      <c r="J21" s="4" t="n"/>
-      <c r="K21" s="4" t="n"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>VINAY</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>BEST</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
-      <c r="H22" s="4" t="n"/>
-      <c r="I22" s="4" t="n"/>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="n"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -3247,109 +2948,91 @@
   </sheetPr>
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
-        <is>
-          <t>Activity Plan  (each row = one combined session group; tick the classes that attend together)</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Activity Plan  (each row = one combined session group)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="B2" s="23" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Allowed Periods</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>LKG</t>
         </is>
       </c>
-      <c r="D2" s="23" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>UKG(A)</t>
         </is>
       </c>
-      <c r="E2" s="23" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>UKG(B)</t>
         </is>
       </c>
-      <c r="F2" s="23" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Class 1(A)</t>
         </is>
       </c>
-      <c r="G2" s="23" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Class 1(B)</t>
         </is>
       </c>
-      <c r="H2" s="23" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Class 2</t>
         </is>
       </c>
-      <c r="I2" s="23" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Class 3</t>
         </is>
       </c>
-      <c r="J2" s="23" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Class 4</t>
         </is>
       </c>
-      <c r="K2" s="23" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Class 5</t>
         </is>
       </c>
-      <c r="L2" s="23" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Class 6</t>
         </is>
       </c>
-      <c r="M2" s="23" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Class 7</t>
         </is>
       </c>
-      <c r="N2" s="23" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Class 8</t>
         </is>
       </c>
-      <c r="O2" s="23" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Class 9</t>
         </is>
       </c>
-      <c r="P2" s="23" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Class 10</t>
         </is>
@@ -3363,7 +3046,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6,7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3425,7 +3108,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6,7</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -3469,19 +3152,59 @@
           <t>Karate</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (19 Jul 2026 23:09)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,27 +29,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002A4D69"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -64,12 +50,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1487,6 +1469,7 @@
           <t>HINDI</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>BIJILI</t>
@@ -1758,6 +1741,11 @@
           <t>K.ESWAR</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1765,6 +1753,15 @@
           <t>PHYSICS</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
@@ -1797,6 +1794,15 @@
           <t>CHEMISTRY</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>K.ESWAR</t>
@@ -1829,6 +1835,15 @@
           <t>BIOLOGY</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>S.GAYATHRI</t>
@@ -1861,6 +1876,12 @@
           <t>SOCIAL</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>R.KAMALA</t>
@@ -1908,6 +1929,9 @@
           <t>COMPUTER</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>VINAY</t>
@@ -1953,6 +1977,8 @@
           <t>VINAY</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1960,6 +1986,9 @@
           <t>G.K</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>CHANDRAKALA</t>
@@ -2005,6 +2034,8 @@
           <t>ESWAR</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2242,6 +2273,9 @@
           <t>Chandini</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2357,6 +2391,10 @@
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2394,6 +2432,10 @@
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2406,6 +2448,9 @@
           <t>MUST</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Leisure</t>
@@ -2478,6 +2523,9 @@
           <t>Leisure</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2490,11 +2538,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2507,11 +2563,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2524,11 +2588,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2541,11 +2613,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2558,11 +2638,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2575,11 +2663,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2592,11 +2688,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2609,11 +2713,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2626,11 +2738,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2643,11 +2763,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2660,11 +2788,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2677,11 +2813,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2694,11 +2838,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2711,11 +2863,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2728,11 +2888,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2745,11 +2913,19 @@
           <t>BEST</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>Lunch Break</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2764,115 +2940,96 @@
   </sheetPr>
   <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Activity Plan  (each row = one combined session group; tick the classes that attend together)</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Activity Plan  (each row = one combined session group)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Allowed Days</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Allowed Periods</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>LKG</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>UKG(A)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>UKG(B)</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Class 1(A)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Class 1(B)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Class 2</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Class 3</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Class 4</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Class 5</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Class 6</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Class 7</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Class 8</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Class 9</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Class 10</t>
         </is>
@@ -2884,7 +3041,11 @@
           <t>P.E.T</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MON,TUE</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>6</t>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (19 Jul 2026 16:15)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -3043,7 +3043,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MON,TUE</t>
+          <t>MON,TUE,WED,THU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3108,7 +3108,11 @@
           <t>P.E.T</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MON,TUE,WED,THU</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>7</t>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (21 Jul 2026 13:42)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -2938,7 +2938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MON,TUE,WED,THU</t>
+          <t>MON,WED,FRI</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3066,36 +3066,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
@@ -3110,7 +3086,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MON,TUE,WED,THU</t>
+          <t>MON,WED,FRI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3121,100 +3097,260 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Karate</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>P.E.T</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TUE,THU</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P.E.T</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TUE,THU</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P.E.T</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TUE,THU</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P.E.T</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MON,SAT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Karate</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>THU</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (21 Jul 2026 13:44)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -3142,22 +3142,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
@@ -3188,22 +3188,22 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
     </row>
@@ -3234,11 +3234,7 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3258,7 +3254,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MON,SAT</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (21 Jul 2026 15:48)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -3129,7 +3129,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TUE,THU</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TUE,THU</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TUE,THU</t>
+          <t>TUE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>THU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (22 Jul 2026 11:07)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -2938,7 +2938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3158,7 +3158,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
@@ -3189,22 +3193,22 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -3235,11 +3239,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3348,6 +3348,49 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P.E.T</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
NRHS: dashboard edit of information workbook (22 Jul 2026 11:19)
</commit_message>
<xml_diff>
--- a/NRHS/Requirements/NRHS_Information.xlsx
+++ b/NRHS/Requirements/NRHS_Information.xlsx
@@ -3209,7 +3209,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3240,11 +3244,7 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3267,19 +3267,35 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3369,7 +3385,11 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
           <t>Yes</t>

</xml_diff>